<commit_message>
act -json in progress
</commit_message>
<xml_diff>
--- a/data/participants_megtusalen.xlsx
+++ b/data/participants_megtusalen.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cristina\repos\megtusalen_validation2026\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROGRAMMING\MATLAB\MEGTUSALEN\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3E5D3F2-39A8-473F-A8B2-78389B326F41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{080D33F9-8F8E-41BD-96E1-D19D1CF72420}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A8CE7551-8922-47F6-B549-E6B85DA15C6C}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{A8CE7551-8922-47F6-B549-E6B85DA15C6C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$BS$730</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$BS$761</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -4856,7 +4856,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -5173,7 +5173,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0FAB02E2-8283-44DB-BC1E-88DE8C1F843E}">
   <dimension ref="A1:BS761"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.7109375" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" customWidth="1"/>
@@ -111472,9 +111472,6 @@
       <c r="B731" t="s">
         <v>1511</v>
       </c>
-      <c r="E731">
-        <v>1</v>
-      </c>
       <c r="BP731">
         <v>0</v>
       </c>
@@ -111904,9 +111901,6 @@
       <c r="B737" t="s">
         <v>1517</v>
       </c>
-      <c r="E737">
-        <v>1</v>
-      </c>
       <c r="BP737">
         <v>0</v>
       </c>
@@ -112941,9 +112935,6 @@
       <c r="B750" t="s">
         <v>1530</v>
       </c>
-      <c r="E750">
-        <v>1</v>
-      </c>
       <c r="AC750">
         <v>48</v>
       </c>
@@ -112973,9 +112964,6 @@
       <c r="B751" t="s">
         <v>1531</v>
       </c>
-      <c r="E751">
-        <v>1</v>
-      </c>
       <c r="AC751">
         <v>24</v>
       </c>
@@ -113005,9 +112993,6 @@
       <c r="B752" t="s">
         <v>1532</v>
       </c>
-      <c r="E752">
-        <v>1</v>
-      </c>
       <c r="BP752">
         <v>0</v>
       </c>
@@ -113391,9 +113376,6 @@
       <c r="B756" t="s">
         <v>1567</v>
       </c>
-      <c r="E756">
-        <v>1</v>
-      </c>
       <c r="BP756">
         <v>0</v>
       </c>
@@ -113505,6 +113487,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BS761" xr:uid="{0FAB02E2-8283-44DB-BC1E-88DE8C1F843E}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>